<commit_message>
added drop 2 & 3 to chords
</commit_message>
<xml_diff>
--- a/hmwebsite/chords/resources/data.xlsx
+++ b/hmwebsite/chords/resources/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\hmon.ir\hmwebsite\chords\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A193A20A-3988-4AAC-985D-EA76E4F6C514}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3DB1100-E3C1-42B0-961C-DB1A83881303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-315" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -441,16 +441,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{91365E13-2B03-42F7-AE33-A38BD1C73E8F}" name="Table1" displayName="Table1" ref="A1:E25" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{91365E13-2B03-42F7-AE33-A38BD1C73E8F}" name="Table1" displayName="Table1" ref="A1:E25" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D9">
     <sortCondition ref="B7:B9"/>
   </sortState>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{3D053E9F-E76F-4AA8-9907-A5D0C5572475}" name="category" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{FE16CA46-A911-4065-9678-BA421DED1555}" name="sortOrder" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{F0E06C2E-5C7A-41B3-85F5-42CB7DE704FF}" name="name" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{D1CEE981-B5D8-4C6E-859D-8E8D7A7B1BEE}" name="path" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{6EC52A06-1682-4082-8D87-A73474C7D0F4}" name="title" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{3D053E9F-E76F-4AA8-9907-A5D0C5572475}" name="category" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{FE16CA46-A911-4065-9678-BA421DED1555}" name="sortOrder" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{F0E06C2E-5C7A-41B3-85F5-42CB7DE704FF}" name="name" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{D1CEE981-B5D8-4C6E-859D-8E8D7A7B1BEE}" name="path" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{6EC52A06-1682-4082-8D87-A73474C7D0F4}" name="title" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>